<commit_message>
Fix govt exclusion: use regex prefix patterns so STATE OF OHIO, IRS TREAS 310 etc all match
</commit_message>
<xml_diff>
--- a/data/Counterparty_Search_Exclusion_List_v9_01_apr.xlsx
+++ b/data/Counterparty_Search_Exclusion_List_v9_01_apr.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B260"/>
+  <dimension ref="A1:B259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3241,7 +3241,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>STATE OF</t>
+          <t>^STATE OF</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -3253,7 +3253,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>IRS TREAS</t>
+          <t>^IRS\b</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -3265,7 +3265,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>IRS</t>
+          <t>^DEPT OF</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -3277,7 +3277,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>DEPT OF REVENUE</t>
+          <t>^US DEPT</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -3289,7 +3289,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>DEPT OF</t>
+          <t>^US TREASURY</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -3301,7 +3301,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>US DEPT</t>
+          <t>^NY STATE</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -3313,7 +3313,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>US TREASURY</t>
+          <t>^VA DEPT</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -3325,7 +3325,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>NY STATE</t>
+          <t>^WVTREASURY</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>VA DEPT</t>
+          <t>^DIVISION OF</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -3349,7 +3349,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>WVTREASURY</t>
+          <t>^CTDOL</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -3361,7 +3361,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>DIVISION OF</t>
+          <t>^TN UI</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -3373,7 +3373,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>CTDOL</t>
+          <t>^GEORGIA DEPART</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -3385,7 +3385,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>TN UI</t>
+          <t>^ST\.? OF</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -3397,7 +3397,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>GEORGIA DEPARTME</t>
+          <t>^SOCIAL SECURITY</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -3409,7 +3409,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>NM BERNALILLO COUNTY</t>
+          <t>^CHILD SUPPORT</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -3421,7 +3421,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>ST. OF MARYLAND</t>
+          <t>^TAX COMMISSION</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -3433,7 +3433,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>SOCIAL SECURITY</t>
+          <t>^FRANCHISE TAX</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -3445,7 +3445,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>CHILD SUPPORT</t>
+          <t>^COMPTROLLER</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -3457,7 +3457,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>TAX COMMISSION</t>
+          <t>^[A-Z]{2}TREASURY</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -3469,22 +3469,10 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>FRANCHISE TAX</t>
+          <t>^[A-Z]{2} DEPT</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
-        <is>
-          <t>Government Agency</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>COMPTROLLER</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
         <is>
           <t>Government Agency</t>
         </is>

</xml_diff>